<commit_message>
mise à jours planning
</commit_message>
<xml_diff>
--- a/documentation/planning.xlsx
+++ b/documentation/planning.xlsx
@@ -226,7 +226,7 @@
     <t>Document Technique</t>
   </si>
   <si>
-    <t>Document Fonctionnelle</t>
+    <t>Document Fonctionnel</t>
   </si>
 </sst>
 </file>
@@ -1149,6 +1149,24 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyProtection="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="12" applyFont="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="12" applyFont="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="11" applyFont="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="11" applyFont="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="12" applyFont="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="11" applyFont="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="168" fontId="0" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
@@ -1159,24 +1177,6 @@
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="166" fontId="7" fillId="0" borderId="3" xfId="9">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="12" applyFont="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="12" applyFont="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="11" applyFont="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="11" applyFont="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="12" applyFont="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="11" applyFont="1" applyFill="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1856,10 +1856,10 @@
       <c r="C3" s="54" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="59">
+      <c r="D3" s="65">
         <v>46095</v>
       </c>
-      <c r="E3" s="59"/>
+      <c r="E3" s="65"/>
     </row>
     <row r="4" spans="1:63" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="30" t="s">
@@ -1869,88 +1869,88 @@
         <v>14</v>
       </c>
       <c r="D4" s="6">
-        <v>1</v>
-      </c>
-      <c r="H4" s="56">
+        <v>3</v>
+      </c>
+      <c r="H4" s="62">
         <f>H5</f>
-        <v>46090</v>
-      </c>
-      <c r="I4" s="57"/>
-      <c r="J4" s="57"/>
-      <c r="K4" s="57"/>
-      <c r="L4" s="57"/>
-      <c r="M4" s="57"/>
-      <c r="N4" s="58"/>
-      <c r="O4" s="56">
+        <v>46104</v>
+      </c>
+      <c r="I4" s="63"/>
+      <c r="J4" s="63"/>
+      <c r="K4" s="63"/>
+      <c r="L4" s="63"/>
+      <c r="M4" s="63"/>
+      <c r="N4" s="64"/>
+      <c r="O4" s="62">
         <f>O5</f>
-        <v>46097</v>
-      </c>
-      <c r="P4" s="57"/>
-      <c r="Q4" s="57"/>
-      <c r="R4" s="57"/>
-      <c r="S4" s="57"/>
-      <c r="T4" s="57"/>
-      <c r="U4" s="58"/>
-      <c r="V4" s="56">
+        <v>46111</v>
+      </c>
+      <c r="P4" s="63"/>
+      <c r="Q4" s="63"/>
+      <c r="R4" s="63"/>
+      <c r="S4" s="63"/>
+      <c r="T4" s="63"/>
+      <c r="U4" s="64"/>
+      <c r="V4" s="62">
         <f>V5</f>
-        <v>46104</v>
-      </c>
-      <c r="W4" s="57"/>
-      <c r="X4" s="57"/>
-      <c r="Y4" s="57"/>
-      <c r="Z4" s="57"/>
-      <c r="AA4" s="57"/>
-      <c r="AB4" s="58"/>
-      <c r="AC4" s="56">
+        <v>46118</v>
+      </c>
+      <c r="W4" s="63"/>
+      <c r="X4" s="63"/>
+      <c r="Y4" s="63"/>
+      <c r="Z4" s="63"/>
+      <c r="AA4" s="63"/>
+      <c r="AB4" s="64"/>
+      <c r="AC4" s="62">
         <f>AC5</f>
-        <v>46111</v>
-      </c>
-      <c r="AD4" s="57"/>
-      <c r="AE4" s="57"/>
-      <c r="AF4" s="57"/>
-      <c r="AG4" s="57"/>
-      <c r="AH4" s="57"/>
-      <c r="AI4" s="58"/>
-      <c r="AJ4" s="56">
+        <v>46125</v>
+      </c>
+      <c r="AD4" s="63"/>
+      <c r="AE4" s="63"/>
+      <c r="AF4" s="63"/>
+      <c r="AG4" s="63"/>
+      <c r="AH4" s="63"/>
+      <c r="AI4" s="64"/>
+      <c r="AJ4" s="62">
         <f>AJ5</f>
-        <v>46118</v>
-      </c>
-      <c r="AK4" s="57"/>
-      <c r="AL4" s="57"/>
-      <c r="AM4" s="57"/>
-      <c r="AN4" s="57"/>
-      <c r="AO4" s="57"/>
-      <c r="AP4" s="58"/>
-      <c r="AQ4" s="56">
+        <v>46132</v>
+      </c>
+      <c r="AK4" s="63"/>
+      <c r="AL4" s="63"/>
+      <c r="AM4" s="63"/>
+      <c r="AN4" s="63"/>
+      <c r="AO4" s="63"/>
+      <c r="AP4" s="64"/>
+      <c r="AQ4" s="62">
         <f>AQ5</f>
-        <v>46125</v>
-      </c>
-      <c r="AR4" s="57"/>
-      <c r="AS4" s="57"/>
-      <c r="AT4" s="57"/>
-      <c r="AU4" s="57"/>
-      <c r="AV4" s="57"/>
-      <c r="AW4" s="58"/>
-      <c r="AX4" s="56">
+        <v>46139</v>
+      </c>
+      <c r="AR4" s="63"/>
+      <c r="AS4" s="63"/>
+      <c r="AT4" s="63"/>
+      <c r="AU4" s="63"/>
+      <c r="AV4" s="63"/>
+      <c r="AW4" s="64"/>
+      <c r="AX4" s="62">
         <f>AX5</f>
-        <v>46132</v>
-      </c>
-      <c r="AY4" s="57"/>
-      <c r="AZ4" s="57"/>
-      <c r="BA4" s="57"/>
-      <c r="BB4" s="57"/>
-      <c r="BC4" s="57"/>
-      <c r="BD4" s="58"/>
-      <c r="BE4" s="56">
+        <v>46146</v>
+      </c>
+      <c r="AY4" s="63"/>
+      <c r="AZ4" s="63"/>
+      <c r="BA4" s="63"/>
+      <c r="BB4" s="63"/>
+      <c r="BC4" s="63"/>
+      <c r="BD4" s="64"/>
+      <c r="BE4" s="62">
         <f>BE5</f>
-        <v>46139</v>
-      </c>
-      <c r="BF4" s="57"/>
-      <c r="BG4" s="57"/>
-      <c r="BH4" s="57"/>
-      <c r="BI4" s="57"/>
-      <c r="BJ4" s="57"/>
-      <c r="BK4" s="58"/>
+        <v>46153</v>
+      </c>
+      <c r="BF4" s="63"/>
+      <c r="BG4" s="63"/>
+      <c r="BH4" s="63"/>
+      <c r="BI4" s="63"/>
+      <c r="BJ4" s="63"/>
+      <c r="BK4" s="64"/>
     </row>
     <row r="5" spans="1:63" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="30" t="s">
@@ -1963,227 +1963,227 @@
       <c r="F5" s="39"/>
       <c r="H5" s="51">
         <f>Début_Projet-WEEKDAY(Début_Projet,1)+2+7*(Semaine_Affichage-1)</f>
-        <v>46090</v>
+        <v>46104</v>
       </c>
       <c r="I5" s="52">
         <f>H5+1</f>
-        <v>46091</v>
+        <v>46105</v>
       </c>
       <c r="J5" s="52">
         <f t="shared" ref="J5:AW5" si="0">I5+1</f>
-        <v>46092</v>
+        <v>46106</v>
       </c>
       <c r="K5" s="52">
         <f t="shared" si="0"/>
-        <v>46093</v>
+        <v>46107</v>
       </c>
       <c r="L5" s="52">
         <f t="shared" si="0"/>
-        <v>46094</v>
+        <v>46108</v>
       </c>
       <c r="M5" s="52">
         <f t="shared" si="0"/>
-        <v>46095</v>
+        <v>46109</v>
       </c>
       <c r="N5" s="53">
         <f t="shared" si="0"/>
-        <v>46096</v>
+        <v>46110</v>
       </c>
       <c r="O5" s="51">
         <f>N5+1</f>
-        <v>46097</v>
+        <v>46111</v>
       </c>
       <c r="P5" s="52">
         <f>O5+1</f>
-        <v>46098</v>
+        <v>46112</v>
       </c>
       <c r="Q5" s="52">
         <f t="shared" si="0"/>
-        <v>46099</v>
+        <v>46113</v>
       </c>
       <c r="R5" s="52">
         <f t="shared" si="0"/>
-        <v>46100</v>
+        <v>46114</v>
       </c>
       <c r="S5" s="52">
         <f t="shared" si="0"/>
-        <v>46101</v>
+        <v>46115</v>
       </c>
       <c r="T5" s="52">
         <f t="shared" si="0"/>
-        <v>46102</v>
+        <v>46116</v>
       </c>
       <c r="U5" s="53">
         <f t="shared" si="0"/>
-        <v>46103</v>
+        <v>46117</v>
       </c>
       <c r="V5" s="51">
         <f>U5+1</f>
-        <v>46104</v>
+        <v>46118</v>
       </c>
       <c r="W5" s="52">
         <f>V5+1</f>
-        <v>46105</v>
+        <v>46119</v>
       </c>
       <c r="X5" s="52">
         <f t="shared" si="0"/>
-        <v>46106</v>
+        <v>46120</v>
       </c>
       <c r="Y5" s="52">
         <f t="shared" si="0"/>
-        <v>46107</v>
+        <v>46121</v>
       </c>
       <c r="Z5" s="52">
         <f t="shared" si="0"/>
-        <v>46108</v>
+        <v>46122</v>
       </c>
       <c r="AA5" s="52">
         <f t="shared" si="0"/>
-        <v>46109</v>
+        <v>46123</v>
       </c>
       <c r="AB5" s="53">
         <f t="shared" si="0"/>
-        <v>46110</v>
+        <v>46124</v>
       </c>
       <c r="AC5" s="51">
         <f>AB5+1</f>
-        <v>46111</v>
+        <v>46125</v>
       </c>
       <c r="AD5" s="52">
         <f>AC5+1</f>
-        <v>46112</v>
+        <v>46126</v>
       </c>
       <c r="AE5" s="52">
         <f t="shared" si="0"/>
-        <v>46113</v>
+        <v>46127</v>
       </c>
       <c r="AF5" s="52">
         <f t="shared" si="0"/>
-        <v>46114</v>
+        <v>46128</v>
       </c>
       <c r="AG5" s="52">
         <f t="shared" si="0"/>
-        <v>46115</v>
+        <v>46129</v>
       </c>
       <c r="AH5" s="52">
         <f t="shared" si="0"/>
-        <v>46116</v>
+        <v>46130</v>
       </c>
       <c r="AI5" s="53">
         <f t="shared" si="0"/>
-        <v>46117</v>
+        <v>46131</v>
       </c>
       <c r="AJ5" s="51">
         <f>AI5+1</f>
-        <v>46118</v>
+        <v>46132</v>
       </c>
       <c r="AK5" s="52">
         <f>AJ5+1</f>
-        <v>46119</v>
+        <v>46133</v>
       </c>
       <c r="AL5" s="52">
         <f t="shared" si="0"/>
-        <v>46120</v>
+        <v>46134</v>
       </c>
       <c r="AM5" s="52">
         <f t="shared" si="0"/>
-        <v>46121</v>
+        <v>46135</v>
       </c>
       <c r="AN5" s="52">
         <f t="shared" si="0"/>
-        <v>46122</v>
+        <v>46136</v>
       </c>
       <c r="AO5" s="52">
         <f t="shared" si="0"/>
-        <v>46123</v>
+        <v>46137</v>
       </c>
       <c r="AP5" s="53">
         <f t="shared" si="0"/>
-        <v>46124</v>
+        <v>46138</v>
       </c>
       <c r="AQ5" s="51">
         <f>AP5+1</f>
-        <v>46125</v>
+        <v>46139</v>
       </c>
       <c r="AR5" s="52">
         <f>AQ5+1</f>
-        <v>46126</v>
+        <v>46140</v>
       </c>
       <c r="AS5" s="52">
         <f t="shared" si="0"/>
-        <v>46127</v>
+        <v>46141</v>
       </c>
       <c r="AT5" s="52">
         <f t="shared" si="0"/>
-        <v>46128</v>
+        <v>46142</v>
       </c>
       <c r="AU5" s="52">
         <f t="shared" si="0"/>
-        <v>46129</v>
+        <v>46143</v>
       </c>
       <c r="AV5" s="52">
         <f t="shared" si="0"/>
-        <v>46130</v>
+        <v>46144</v>
       </c>
       <c r="AW5" s="53">
         <f t="shared" si="0"/>
-        <v>46131</v>
+        <v>46145</v>
       </c>
       <c r="AX5" s="51">
         <f>AW5+1</f>
-        <v>46132</v>
+        <v>46146</v>
       </c>
       <c r="AY5" s="52">
         <f>AX5+1</f>
-        <v>46133</v>
+        <v>46147</v>
       </c>
       <c r="AZ5" s="52">
         <f t="shared" ref="AZ5:BD5" si="1">AY5+1</f>
-        <v>46134</v>
+        <v>46148</v>
       </c>
       <c r="BA5" s="52">
         <f t="shared" si="1"/>
-        <v>46135</v>
+        <v>46149</v>
       </c>
       <c r="BB5" s="52">
         <f t="shared" si="1"/>
-        <v>46136</v>
+        <v>46150</v>
       </c>
       <c r="BC5" s="52">
         <f t="shared" si="1"/>
-        <v>46137</v>
+        <v>46151</v>
       </c>
       <c r="BD5" s="53">
         <f t="shared" si="1"/>
-        <v>46138</v>
+        <v>46152</v>
       </c>
       <c r="BE5" s="51">
         <f>BD5+1</f>
-        <v>46139</v>
+        <v>46153</v>
       </c>
       <c r="BF5" s="52">
         <f>BE5+1</f>
-        <v>46140</v>
+        <v>46154</v>
       </c>
       <c r="BG5" s="52">
         <f t="shared" ref="BG5:BK5" si="2">BF5+1</f>
-        <v>46141</v>
+        <v>46155</v>
       </c>
       <c r="BH5" s="52">
         <f t="shared" si="2"/>
-        <v>46142</v>
+        <v>46156</v>
       </c>
       <c r="BI5" s="52">
         <f t="shared" si="2"/>
-        <v>46143</v>
+        <v>46157</v>
       </c>
       <c r="BJ5" s="52">
         <f t="shared" si="2"/>
-        <v>46144</v>
+        <v>46158</v>
       </c>
       <c r="BK5" s="53">
         <f t="shared" si="2"/>
-        <v>46145</v>
+        <v>46159</v>
       </c>
     </row>
     <row r="6" spans="1:63" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -2574,10 +2574,10 @@
       <c r="A9" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="60" t="s">
+      <c r="B9" s="56" t="s">
         <v>34</v>
       </c>
-      <c r="C9" s="62" t="s">
+      <c r="C9" s="58" t="s">
         <v>44</v>
       </c>
       <c r="D9" s="44">
@@ -2654,10 +2654,10 @@
       <c r="A10" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="60" t="s">
+      <c r="B10" s="56" t="s">
         <v>37</v>
       </c>
-      <c r="C10" s="62" t="s">
+      <c r="C10" s="58" t="s">
         <v>45</v>
       </c>
       <c r="D10" s="44">
@@ -2732,10 +2732,10 @@
     </row>
     <row r="11" spans="1:63" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="29"/>
-      <c r="B11" s="60" t="s">
+      <c r="B11" s="56" t="s">
         <v>38</v>
       </c>
-      <c r="C11" s="62" t="s">
+      <c r="C11" s="58" t="s">
         <v>45</v>
       </c>
       <c r="D11" s="44">
@@ -2810,10 +2810,10 @@
     </row>
     <row r="12" spans="1:63" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="29"/>
-      <c r="B12" s="60" t="s">
+      <c r="B12" s="56" t="s">
         <v>42</v>
       </c>
-      <c r="C12" s="62" t="s">
+      <c r="C12" s="58" t="s">
         <v>43</v>
       </c>
       <c r="D12" s="44">
@@ -2956,10 +2956,10 @@
     </row>
     <row r="14" spans="1:63" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="30"/>
-      <c r="B14" s="61" t="s">
+      <c r="B14" s="57" t="s">
         <v>39</v>
       </c>
-      <c r="C14" s="63" t="s">
+      <c r="C14" s="59" t="s">
         <v>43</v>
       </c>
       <c r="D14" s="47">
@@ -3034,10 +3034,10 @@
     </row>
     <row r="15" spans="1:63" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="29"/>
-      <c r="B15" s="61" t="s">
+      <c r="B15" s="57" t="s">
         <v>40</v>
       </c>
-      <c r="C15" s="63" t="s">
+      <c r="C15" s="59" t="s">
         <v>46</v>
       </c>
       <c r="D15" s="47">
@@ -3111,10 +3111,10 @@
     </row>
     <row r="16" spans="1:63" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="29"/>
-      <c r="B16" s="61" t="s">
+      <c r="B16" s="57" t="s">
         <v>41</v>
       </c>
-      <c r="C16" s="63" t="s">
+      <c r="C16" s="59" t="s">
         <v>46</v>
       </c>
       <c r="D16" s="47">
@@ -3258,23 +3258,23 @@
     </row>
     <row r="18" spans="1:63" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="29"/>
-      <c r="B18" s="64" t="s">
+      <c r="B18" s="60" t="s">
         <v>48</v>
       </c>
-      <c r="C18" s="65" t="s">
+      <c r="C18" s="61" t="s">
         <v>46</v>
       </c>
       <c r="D18" s="50">
         <v>46129</v>
       </c>
       <c r="E18" s="50">
-        <f>D18+27</f>
-        <v>46156</v>
+        <f>D18+34</f>
+        <v>46163</v>
       </c>
       <c r="F18" s="12"/>
-      <c r="G18" s="12" t="e">
+      <c r="G18" s="12">
         <f t="shared" si="5"/>
-        <v>#REF!</v>
+        <v>35</v>
       </c>
       <c r="H18" s="16"/>
       <c r="I18" s="16"/>
@@ -3335,10 +3335,10 @@
     </row>
     <row r="19" spans="1:63" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="29"/>
-      <c r="B19" s="64" t="s">
+      <c r="B19" s="60" t="s">
         <v>49</v>
       </c>
-      <c r="C19" s="65" t="s">
+      <c r="C19" s="61" t="s">
         <v>46</v>
       </c>
       <c r="D19" s="50">
@@ -3573,23 +3573,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Url xsi:nil="true"/>
-      <Description xsi:nil="true"/>
-    </Image>
-    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
-    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </ImageTagsTaxHTField>
-    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
-    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3881,29 +3870,29 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Url xsi:nil="true"/>
+      <Description xsi:nil="true"/>
+    </Image>
+    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
+    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </ImageTagsTaxHTField>
+    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
+    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AC3AD2E1-977A-4D4F-8EE8-D64B5FFADF75}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E4A34E49-7289-4AEA-9593-4F55E04ADB10}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="16c05727-aa75-4e4a-9b5f-8a80a1165891"/>
-    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
-    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -3930,9 +3919,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E4A34E49-7289-4AEA-9593-4F55E04ADB10}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AC3AD2E1-977A-4D4F-8EE8-D64B5FFADF75}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="16c05727-aa75-4e4a-9b5f-8a80a1165891"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>